<commit_message>
docs: add review-effort benchmarks and rate-base worksheet
Add knowledge/review-effort-benchmarks.md: external requirements-review
speed norms (Gilb/Graham, Wiegers), a rescale to a 10-page ТЗ, and an
assumption-based effort decomposition model, cross-checked against the
economics.md hourly assumption without treating the match as proof.

Register S-28/S-29 sources and link the new doc from README.md and
knowledge/sources.md. Update МТС_AI_Reviwe.xlsx with the "База ставок"
worksheet backing the hourly rates. Ignore Office lock files (~$*.xls*
etc.) so they stop getting staged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/МТС_AI_Reviwe.xlsx
+++ b/МТС_AI_Reviwe.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danil\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ITMO\GIT\MTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59151740-7CF9-494D-936F-CB71FC689507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28274051-028B-4247-ADD3-133150212C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="База ставок" sheetId="4" r:id="rId7"/>
-    <sheet name="Исходные данные" sheetId="3" r:id="rId1"/>
-    <sheet name="Экономический эффект" sheetId="1" r:id="rId2"/>
+    <sheet name="База ставок" sheetId="4" r:id="rId1"/>
+    <sheet name="Исходные данные" sheetId="3" r:id="rId2"/>
+    <sheet name="Экономический эффект" sheetId="1" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
   <si>
     <t>Показатель</t>
   </si>
@@ -84,6 +84,54 @@
   </si>
   <si>
     <t>Сокращение трудозатрат разработчика</t>
+  </si>
+  <si>
+    <t>Основание</t>
+  </si>
+  <si>
+    <t>Медианная зарплата Middle системного аналитика, ₽/мес до НДФЛ</t>
+  </si>
+  <si>
+    <t>Хабр Карьера, страница «Системный аналитик, Middle», 1 219 анкет; сверено 2026-09-05</t>
+  </si>
+  <si>
+    <t>Медианная зарплата Middle бэкенд-разработчика, ₽/мес до НДФЛ</t>
+  </si>
+  <si>
+    <t>Хабр Карьера, страница «Бэкенд разработчик, Middle», 3 449 анкет; сверено 2026-09-05</t>
+  </si>
+  <si>
+    <t>Ставка страховых взносов работодателя</t>
+  </si>
+  <si>
+    <t>Единый тариф 30 % до предельной базы; для аккредитованной ИТ-компании ставится 7,6 %</t>
+  </si>
+  <si>
+    <t>Годовая норма рабочего времени, ч</t>
+  </si>
+  <si>
+    <t>Производственный календарь 2026, 40-часовая неделя, 247 рабочих дней</t>
+  </si>
+  <si>
+    <t>Среднемесячная норма рабочего времени, ч</t>
+  </si>
+  <si>
+    <t>Годовая норма, делённая на 12</t>
+  </si>
+  <si>
+    <t>Зарплата с взносами, делённая на месячную норму часов</t>
+  </si>
+  <si>
+    <t>Стоимость часа = медианная зарплата × (1 + ставка взносов) ÷ среднемесячная норма часов. Это полная стоимость часа для работодателя, а не выплата сотруднику.</t>
+  </si>
+  <si>
+    <t>Премии, накладные расходы, отпускные сверх нормы и региональные надбавки в расчёт не входят.</t>
+  </si>
+  <si>
+    <t>Значения являются рыночными медианами, а не подтверждёнными ставками MTS. Разбор и ограничения — knowledge/economics.md.</t>
+  </si>
+  <si>
+    <t>Эффект в год (на одну команду)</t>
   </si>
 </sst>
 </file>
@@ -428,7 +476,128 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D588A51-B44C-4635-84ED-730A5CFCC9C3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{723B0AB1-CE2B-4A92-AFB4-94462C4942C1}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="52" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="72" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2">
+        <v>204441</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2">
+        <v>220833</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5">
+        <v>1972</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="5">
+        <f>B5/12</f>
+        <v>164.33333333333334</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <f>ROUND(B2*(1+B4)/B6,0)</f>
+        <v>1617</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <f>ROUND(B3*(1+B4)/B6,0)</f>
+        <v>1747</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A67E427B-1D16-4F82-AE67-3B119B0EB4C3}">
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -482,7 +651,7 @@
       </c>
       <c r="B6" s="2">
         <f>'База ставок'!B7</f>
-        <v>1617.0</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -491,7 +660,7 @@
       </c>
       <c r="B7" s="2">
         <f>'База ставок'!B8</f>
-        <v>1747.0</v>
+        <v>1747</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -499,7 +668,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="1">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -507,141 +676,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="32" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2">
-        <v>10</v>
-      </c>
-      <c r="C2">
-        <f>B2</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="C3" s="1">
-        <f>B3*0.2</f>
-        <v>8.0000000000000016E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" s="5">
-        <f>(1-'Исходные данные'!B8)*B4</f>
-        <v>0.39999999999999991</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5" s="5">
-        <f>(1-'Исходные данные'!B9)*B5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="2">
-        <f>'Исходные данные'!B6</f>
-        <v>1617.0</v>
-      </c>
-      <c r="C6" s="2">
-        <f>B6</f>
-        <v>1617.0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="2">
-        <f>'Исходные данные'!B7</f>
-        <v>1747.0</v>
-      </c>
-      <c r="C7" s="2">
-        <f>B7</f>
-        <v>1747.0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="3">
-        <f>B5*B7+B4*B6</f>
-        <v>4981.0</v>
-      </c>
-      <c r="C8" s="3">
-        <f>C5*C7+C4*C6</f>
-        <v>646.7999999999998</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="3">
-        <f>B2*B3*B8</f>
-        <v>19924.0</v>
-      </c>
-      <c r="C9" s="3">
-        <f>C2*C3*C8</f>
-        <v>517.4399999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="3">
-        <f>B9-C9</f>
-        <v>19406.56</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -650,159 +685,141 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4E748ED-1089-4701-A8B7-34B4A30F65C0}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="52" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="72" customWidth="1"/>
+    <col min="1" max="1" width="32" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Показатель</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Значение</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основание</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Медианная зарплата Middle системного аналитика, ₽/мес до НДФЛ</t>
-        </is>
-      </c>
-      <c r="B2" s="2">
-        <v>204441.0</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Хабр Карьера, страница «Системный аналитик, Middle», 1 219 анкет; сверено 2026-09-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Медианная зарплата Middle бэкенд-разработчика, ₽/мес до НДФЛ</t>
-        </is>
-      </c>
-      <c r="B3" s="2">
-        <v>220833.0</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Хабр Карьера, страница «Бэкенд разработчик, Middle», 3 449 анкет; сверено 2026-09-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ставка страховых взносов работодателя</t>
-        </is>
-      </c>
-      <c r="B4" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Единый тариф 30 % до предельной базы; для аккредитованной ИТ-компании ставится 7,6 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Годовая норма рабочего времени, ч</t>
-        </is>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <f>B2</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="5">
+        <f>(1-'Исходные данные'!B8)*B4</f>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>11</v>
       </c>
       <c r="B5">
-        <v>1972.0</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Производственный календарь 2026, 40-часовая неделя, 247 рабочих дней</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Среднемесячная норма рабочего времени, ч</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>B5/12</f>
-        <v>164.33333333333334</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Годовая норма, делённая на 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Стоимость часа аналитика</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <f>(1-'Исходные данные'!B9)*B5</f>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2">
+        <f>'Исходные данные'!B6</f>
+        <v>1617</v>
+      </c>
+      <c r="C6" s="2">
+        <f>B6</f>
+        <v>1617</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>7</v>
       </c>
       <c r="B7" s="2">
-        <f>ROUND(B2*(1+B4)/B6,0)</f>
-        <v>1617.0</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Зарплата с взносами, делённая на месячную норму часов</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Стоимость часа разработчика</t>
-        </is>
-      </c>
-      <c r="B8" s="2">
-        <f>ROUND(B3*(1+B4)/B6,0)</f>
-        <v>1747.0</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Зарплата с взносами, делённая на месячную норму часов</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Стоимость часа = медианная зарплата × (1 + ставка взносов) ÷ среднемесячная норма часов. Это полная стоимость часа для работодателя, а не выплата сотруднику.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Премии, накладные расходы, отпускные сверх нормы и региональные надбавки в расчёт не входят.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Значения являются рыночными медианами, а не подтверждёнными ставками MTS. Разбор и ограничения — knowledge/economics.md.</t>
-        </is>
+        <f>'Исходные данные'!B7</f>
+        <v>1747</v>
+      </c>
+      <c r="C7" s="2">
+        <f>B7</f>
+        <v>1747</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="3">
+        <f>B5*B7+B4*B6</f>
+        <v>4981</v>
+      </c>
+      <c r="C8" s="3">
+        <f>C5*C7+C4*C6</f>
+        <v>1992.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="3">
+        <f>B2*B3*B8</f>
+        <v>19924</v>
+      </c>
+      <c r="C9" s="3">
+        <f>C2*C3*C8</f>
+        <v>7969.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="3">
+        <f>B9-C9</f>
+        <v>11954.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="3">
+        <f>C10*12</f>
+        <v>143452.79999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>